<commit_message>
Hooked Shorts Excel 任务 sheet 改名为 HookedShorts任务。
与其他工具的「任务列表」区分，读取逻辑兼容旧表名。

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/未来管理系统批量脚本工具/ad-automation3.0/data/tasks-v3.0.xlsx
+++ b/未来管理系统批量脚本工具/ad-automation3.0/data/tasks-v3.0.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="任务列表" sheetId="1" r:id="rId1"/>
+    <sheet name="HookedShorts任务" sheetId="1" r:id="rId1"/>
     <sheet name="字段说明" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
@@ -399,34 +399,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z6"/>
-  <cols>
-    <col min="1" max="1" width="6.83203125" customWidth="1"/>
-    <col min="2" max="2" width="8.83203125" customWidth="1"/>
-    <col min="3" max="3" width="22.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="18.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-    <col min="7" max="7" width="12.83203125" customWidth="1"/>
-    <col min="8" max="8" width="14.83203125" customWidth="1"/>
-    <col min="9" max="9" width="30.83203125" customWidth="1"/>
-    <col min="10" max="10" width="14.83203125" customWidth="1"/>
-    <col min="11" max="11" width="22.83203125" customWidth="1"/>
-    <col min="12" max="12" width="35.83203125" customWidth="1"/>
-    <col min="13" max="13" width="10.83203125" customWidth="1"/>
-    <col min="14" max="14" width="16.83203125" customWidth="1"/>
-    <col min="15" max="15" width="8.83203125" customWidth="1"/>
-    <col min="16" max="16" width="10.83203125" customWidth="1"/>
-    <col min="17" max="17" width="6.83203125" customWidth="1"/>
-    <col min="18" max="18" width="12.83203125" customWidth="1"/>
-    <col min="19" max="19" width="10.83203125" customWidth="1"/>
-    <col min="20" max="20" width="6.83203125" customWidth="1"/>
-    <col min="21" max="21" width="10.83203125" customWidth="1"/>
-    <col min="22" max="22" width="10.83203125" customWidth="1"/>
-    <col min="23" max="23" width="10.83203125" customWidth="1"/>
-    <col min="24" max="24" width="8.83203125" customWidth="1"/>
-    <col min="25" max="25" width="18.83203125" customWidth="1"/>
-    <col min="26" max="26" width="10.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -920,12 +892,6 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D27"/>
-  <cols>
-    <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="50.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="30.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>